<commit_message>
Fix SonarQube Report hyperlinks
</commit_message>
<xml_diff>
--- a/report/SonarQube Report.xlsx
+++ b/report/SonarQube Report.xlsx
@@ -126,7 +126,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,12 +164,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -217,40 +211,28 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -415,9 +397,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>87480</xdr:colOff>
+      <xdr:colOff>87120</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>65880</xdr:rowOff>
+      <xdr:rowOff>65520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -431,7 +413,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="17967960" cy="8209800"/>
+          <a:ext cx="17917920" cy="8209440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -457,9 +439,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -473,7 +455,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -499,9 +481,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -515,7 +497,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -541,9 +523,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -557,7 +539,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -583,9 +565,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -599,7 +581,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -625,9 +607,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -641,7 +623,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -667,9 +649,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -683,7 +665,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -709,9 +691,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -725,7 +707,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -751,9 +733,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -767,7 +749,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -793,9 +775,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -809,7 +791,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -835,9 +817,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -851,7 +833,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -877,9 +859,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>87480</xdr:colOff>
+      <xdr:colOff>87120</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>65880</xdr:rowOff>
+      <xdr:rowOff>65520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -893,7 +875,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="17967960" cy="8209800"/>
+          <a:ext cx="17917920" cy="8209440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -919,9 +901,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -935,7 +917,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -961,9 +943,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -977,7 +959,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1003,9 +985,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>247320</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>114480</xdr:rowOff>
+      <xdr:colOff>246960</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>148680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1019,7 +1001,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128880" cy="8242560"/>
+          <a:ext cx="18100800" cy="8210520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1045,9 +1027,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>87480</xdr:colOff>
+      <xdr:colOff>87120</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>65880</xdr:rowOff>
+      <xdr:rowOff>65520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1061,7 +1043,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="17967960" cy="8209800"/>
+          <a:ext cx="17917920" cy="8209440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1087,9 +1069,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1103,7 +1085,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1129,9 +1111,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1145,7 +1127,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1171,9 +1153,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1187,7 +1169,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1213,9 +1195,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1229,7 +1211,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1255,9 +1237,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1271,7 +1253,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1297,9 +1279,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>246960</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5040</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1313,7 +1295,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="18128520" cy="8242200"/>
+          <a:ext cx="18100440" cy="8062920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1518,429 +1500,429 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="23.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="13.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="77.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="77.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C19" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D28" s="4"/>
+      <c r="D28" s="3"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D6:D28">
@@ -1961,25 +1943,25 @@
     <hyperlink ref="C6" location="'1'!A1" display="#'1'.A1"/>
     <hyperlink ref="C7" location="'2'!A1" display="#'2'.A1"/>
     <hyperlink ref="C8" location="'3'!A1" display="#'3'.A1"/>
-    <hyperlink ref="C9" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C10" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C11" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C12" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C13" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C14" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C15" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C16" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C17" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C18" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C19" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C20" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C21" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C22" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C23" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C24" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C25" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C26" location="'1'!A1" display="#'1'.A1"/>
-    <hyperlink ref="C27" location="'1'!A1" display="#'1'.A1"/>
+    <hyperlink ref="C9" location="'4'!A1" display="#'4'.A1"/>
+    <hyperlink ref="C10" location="'5'!A1" display="#'5'.A1"/>
+    <hyperlink ref="C11" location="'6'!A1" display="#'6'.A1"/>
+    <hyperlink ref="C12" location="'7'!A1" display="#'7'.A1"/>
+    <hyperlink ref="C13" location="'8'!A1" display="#'8'.A1"/>
+    <hyperlink ref="C14" location="'9'!A1" display="#'9'.A1"/>
+    <hyperlink ref="C15" location="'10'!A1" display="#'10'.A1"/>
+    <hyperlink ref="C16" location="'11'!A1" display="#'11'.A1"/>
+    <hyperlink ref="C17" location="'12'!A1" display="#'12'.A1"/>
+    <hyperlink ref="C18" location="'13'!A1" display="#'13'.A1"/>
+    <hyperlink ref="C19" location="'14'!A1" display="#'14'.A1"/>
+    <hyperlink ref="C20" location="'15'!A1" display="#'15'.A1"/>
+    <hyperlink ref="C21" location="'16'!A1" display="#'16'.A1"/>
+    <hyperlink ref="C22" location="'17'!A1" display="#'17'.A1"/>
+    <hyperlink ref="C23" location="'18'!A1" display="#'18'.A1"/>
+    <hyperlink ref="C24" location="'19'!A1" display="#'19'.A1"/>
+    <hyperlink ref="C25" location="'20'!A1" display="#'20'.A1"/>
+    <hyperlink ref="C26" location="'21'!A1" display="#'21'.A1"/>
+    <hyperlink ref="C27" location="'22'!A1" display="#'22'.A1"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2000,7 +1982,949 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2065,13 +2989,51 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2121,9 +3083,9 @@
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -2136,13 +3098,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2192,9 +3154,9 @@
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -2207,13 +3169,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2263,9 +3225,9 @@
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -2278,13 +3240,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2334,9 +3296,9 @@
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -2349,13 +3311,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2405,937 +3367,9 @@
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>